<commit_message>
Cambio rural por densidad y otros cambios
</commit_message>
<xml_diff>
--- a/Output/individual_characteristics_lpm_logit_specs.xlsx
+++ b/Output/individual_characteristics_lpm_logit_specs.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">spec</t>
   </si>
@@ -68,51 +68,36 @@
     <t xml:space="preserve">0.053*** (0.011)</t>
   </si>
   <si>
-    <t xml:space="preserve">rural</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.047 (0.033)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.040 (0.032)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.050** (0.024)</t>
+    <t xml:space="preserve">desempleado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.030 (0.027)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.040 (0.024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.035 (0.023)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">en_pareja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.051*** (0.011)</t>
   </si>
   <si>
     <t xml:space="preserve">-**</t>
   </si>
   <si>
-    <t xml:space="preserve">desempleado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.029 (0.027)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.039 (0.025)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.033 (0.024)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">en_pareja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.050*** (0.011)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.044*** (0.009)</t>
   </si>
   <si>
@@ -122,13 +107,13 @@
     <t xml:space="preserve">secundaria_completa_o_mas</t>
   </si>
   <si>
-    <t xml:space="preserve">0.025** (0.011)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.020** (0.009)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.031*** (0.010)</t>
+    <t xml:space="preserve">0.026** (0.011)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.021** (0.010)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.032*** (0.010)</t>
   </si>
   <si>
     <t xml:space="preserve">izq_der</t>
@@ -143,10 +128,10 @@
     <t xml:space="preserve">0.018 (0.013)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.025* (0.013)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.017 (0.013)</t>
+    <t xml:space="preserve">0.025** (0.013)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.016 (0.013)</t>
   </si>
   <si>
     <t xml:space="preserve">voto_blanco_nulo</t>
@@ -155,7 +140,7 @@
     <t xml:space="preserve">0.036** (0.015)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.037*** (0.013)</t>
+    <t xml:space="preserve">0.036*** (0.013)</t>
   </si>
 </sst>
 </file>
@@ -655,7 +640,7 @@
         <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E9" t="n">
         <v>6155</v>
@@ -672,10 +657,10 @@
         <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E10" t="n">
         <v>5641</v>
@@ -689,13 +674,13 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E11" t="n">
         <v>4966</v>
@@ -709,13 +694,13 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" t="s">
         <v>27</v>
-      </c>
-      <c r="D12" t="s">
-        <v>28</v>
       </c>
       <c r="E12" t="n">
         <v>6155</v>
@@ -729,13 +714,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
         <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E13" t="n">
         <v>5641</v>
@@ -749,13 +734,13 @@
         <v>6</v>
       </c>
       <c r="B14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" t="s">
         <v>31</v>
       </c>
-      <c r="C14" t="s">
-        <v>32</v>
-      </c>
       <c r="D14" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E14" t="n">
         <v>4966</v>
@@ -769,13 +754,13 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E15" t="n">
         <v>6155</v>
@@ -789,13 +774,13 @@
         <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D16" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E16" t="n">
         <v>5641</v>
@@ -809,13 +794,13 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" t="s">
         <v>35</v>
       </c>
-      <c r="C17" t="s">
-        <v>36</v>
-      </c>
       <c r="D17" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E17" t="n">
         <v>4966</v>
@@ -829,13 +814,13 @@
         <v>10</v>
       </c>
       <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" t="s">
         <v>35</v>
       </c>
-      <c r="C18" t="s">
-        <v>37</v>
-      </c>
       <c r="D18" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E18" t="n">
         <v>6155</v>
@@ -846,62 +831,62 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D19" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E19" t="n">
-        <v>5641</v>
+        <v>4966</v>
       </c>
       <c r="F19" t="n">
-        <v>5641</v>
+        <v>4966</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D20" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E20" t="n">
-        <v>4966</v>
+        <v>6155</v>
       </c>
       <c r="F20" t="n">
-        <v>4966</v>
+        <v>6155</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" t="s">
         <v>39</v>
       </c>
-      <c r="C21" t="s">
-        <v>40</v>
-      </c>
       <c r="D21" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E21" t="n">
-        <v>6155</v>
+        <v>5641</v>
       </c>
       <c r="F21" t="n">
-        <v>6155</v>
+        <v>5641</v>
       </c>
     </row>
     <row r="22">
@@ -909,13 +894,13 @@
         <v>6</v>
       </c>
       <c r="B22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" t="s">
         <v>41</v>
       </c>
-      <c r="C22" t="s">
-        <v>42</v>
-      </c>
       <c r="D22" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E22" t="n">
         <v>4966</v>
@@ -926,81 +911,21 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D23" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="E23" t="n">
-        <v>6155</v>
+        <v>5641</v>
       </c>
       <c r="F23" t="n">
-        <v>6155</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s">
-        <v>12</v>
-      </c>
-      <c r="B24" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" t="s">
-        <v>26</v>
-      </c>
-      <c r="E24" t="n">
-        <v>5641</v>
-      </c>
-      <c r="F24" t="n">
-        <v>5641</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" t="s">
-        <v>46</v>
-      </c>
-      <c r="D25" t="s">
-        <v>28</v>
-      </c>
-      <c r="E25" t="n">
-        <v>4966</v>
-      </c>
-      <c r="F25" t="n">
-        <v>4966</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s">
-        <v>12</v>
-      </c>
-      <c r="B26" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" t="s">
-        <v>47</v>
-      </c>
-      <c r="D26" t="s">
-        <v>15</v>
-      </c>
-      <c r="E26" t="n">
-        <v>5641</v>
-      </c>
-      <c r="F26" t="n">
         <v>5641</v>
       </c>
     </row>

</xml_diff>